<commit_message>
fixed peer coding visibility
</commit_message>
<xml_diff>
--- a/data/demo.xlsx
+++ b/data/demo.xlsx
@@ -414,7 +414,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="2">
-        <v>46029</v>
+        <v>46034</v>
       </c>
     </row>
     <row r="3">
@@ -438,7 +438,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="2">
-        <v>46028</v>
+        <v>46033</v>
       </c>
     </row>
     <row r="4">
@@ -462,7 +462,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>46027</v>
+        <v>46032</v>
       </c>
     </row>
     <row r="5">
@@ -486,7 +486,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <v>46026</v>
+        <v>46031</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         <v>5.5</v>
       </c>
       <c r="F6" s="2">
-        <v>46025</v>
+        <v>46030</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="2">
-        <v>46024</v>
+        <v>46029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>